<commit_message>
Updated template and tests
</commit_message>
<xml_diff>
--- a/src/clients/ApplicationTracker.Angular/public/templates/ApplicationRecords_Import_Template.xlsx
+++ b/src/clients/ApplicationTracker.Angular/public/templates/ApplicationRecords_Import_Template.xlsx
@@ -563,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -760,223 +760,255 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="8" customHeight="1"/>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="11" ht="8" customHeight="1">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Description (F)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Any text</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Full-stack engineer role requiring React and Node.js experience</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Job posting description; leave blank if none. Max 20,000 characters.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1"/>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Rules and Validation</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="12" t="inlineStr">
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>• CompanyName and AppliedDate are required for every row — rows missing either will be skipped with an error.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="13" t="inlineStr">
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>• Status must be the text name (Applied, Interviewing, Offered, Rejected, Withdrawn). Numeric values (0–4) are rejected.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="12" t="inlineStr">
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>• Duplicate detection: if a record with the same CompanyName + PostingUrl already exists in your account it will be skipped.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="13" t="inlineStr">
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">  If no PostingUrl is provided, CompanyName + AppliedDate is used for duplicate detection instead.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="12" t="inlineStr">
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>• PostingUrl must be a valid http:// or https:// URL if provided. Partial URLs (e.g. "careers.google.com") will be rejected.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="13" t="inlineStr">
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="13" t="inlineStr">
         <is>
           <t>• Future dates are not accepted for AppliedDate.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>• Extra columns beyond column E are ignored.</t>
-        </is>
-      </c>
-    </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="13" t="inlineStr">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>• Extra columns beyond column F are ignored.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="8" customHeight="1">
+      <c r="A21" s="13" t="inlineStr">
         <is>
           <t>• Do not modify or delete the header row (row 1) on the Data sheet.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="8" customHeight="1"/>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="22" ht="20" customHeight="1"/>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Example Rows (for reference only — do not paste into the Data sheet)</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="14" t="inlineStr">
+    <row r="24" ht="16" customHeight="1">
+      <c r="A24" s="14" t="inlineStr">
         <is>
           <t>CompanyName</t>
         </is>
       </c>
-      <c r="B23" s="14" t="inlineStr">
+      <c r="B24" s="14" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="C23" s="14" t="inlineStr">
+      <c r="C24" s="14" t="inlineStr">
         <is>
           <t>AppliedDate</t>
         </is>
       </c>
-      <c r="D23" s="14" t="inlineStr">
+      <c r="D24" s="14" t="inlineStr">
         <is>
           <t>PostingUrl</t>
         </is>
       </c>
-      <c r="E23" s="14" t="inlineStr">
+      <c r="E24" s="14" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-    </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="15" t="inlineStr">
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="16" customHeight="1">
+      <c r="A25" s="15" t="inlineStr">
         <is>
           <t>Google</t>
         </is>
       </c>
-      <c r="B24" s="15" t="inlineStr">
+      <c r="B25" s="15" t="inlineStr">
         <is>
           <t>Applied</t>
         </is>
       </c>
-      <c r="C24" s="15" t="inlineStr">
+      <c r="C25" s="15" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="D24" s="15" t="inlineStr">
+      <c r="D25" s="15" t="inlineStr">
         <is>
           <t>https://careers.google.com/jobs/123</t>
         </is>
       </c>
-      <c r="E24" s="15" t="inlineStr"/>
-    </row>
-    <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="16" t="inlineStr">
+      <c r="E25" s="15" t="inlineStr"/>
+    </row>
+    <row r="26" ht="16" customHeight="1">
+      <c r="A26" s="16" t="inlineStr">
         <is>
           <t>Microsoft</t>
         </is>
       </c>
-      <c r="B25" s="16" t="inlineStr">
+      <c r="B26" s="16" t="inlineStr">
         <is>
           <t>Interviewing</t>
         </is>
       </c>
-      <c r="C25" s="16" t="inlineStr">
+      <c r="C26" s="16" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
       </c>
-      <c r="D25" s="16" t="inlineStr">
+      <c r="D26" s="16" t="inlineStr">
         <is>
           <t>https://careers.microsoft.com/job/456</t>
         </is>
       </c>
-      <c r="E25" s="16" t="inlineStr">
+      <c r="E26" s="16" t="inlineStr">
         <is>
           <t>Phone screen passed</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="15" t="inlineStr">
+    <row r="27" ht="16" customHeight="1">
+      <c r="A27" s="15" t="inlineStr">
         <is>
           <t>Airbnb</t>
         </is>
       </c>
-      <c r="B26" s="15" t="inlineStr">
+      <c r="B27" s="15" t="inlineStr">
         <is>
           <t>Offered</t>
         </is>
       </c>
-      <c r="C26" s="15" t="inlineStr">
+      <c r="C27" s="15" t="inlineStr">
         <is>
           <t>2026-04-10</t>
         </is>
       </c>
-      <c r="D26" s="15" t="inlineStr"/>
-      <c r="E26" s="15" t="inlineStr">
+      <c r="D27" s="15" t="inlineStr"/>
+      <c r="E27" s="15" t="inlineStr">
         <is>
           <t>Offer expires June 30</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="16" t="inlineStr">
+    <row r="28" ht="16" customHeight="1">
+      <c r="A28" s="16" t="inlineStr">
         <is>
           <t>Amazon</t>
         </is>
       </c>
-      <c r="B27" s="16" t="inlineStr">
+      <c r="B28" s="16" t="inlineStr">
         <is>
           <t>Rejected</t>
         </is>
       </c>
-      <c r="C27" s="16" t="inlineStr">
+      <c r="C28" s="16" t="inlineStr">
         <is>
           <t>2026-03-01</t>
         </is>
       </c>
-      <c r="D27" s="16" t="inlineStr">
+      <c r="D28" s="16" t="inlineStr">
         <is>
           <t>https://amazon.jobs/en/jobs/789</t>
         </is>
       </c>
-      <c r="E27" s="16" t="inlineStr">
+      <c r="E28" s="16" t="inlineStr">
         <is>
           <t>Did not pass bar raiser</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="15" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="15" t="inlineStr">
         <is>
           <t>Startup Co</t>
         </is>
       </c>
-      <c r="B28" s="15" t="inlineStr">
+      <c r="B29" s="15" t="inlineStr">
         <is>
           <t>Withdrawn</t>
         </is>
       </c>
-      <c r="C28" s="15" t="inlineStr">
+      <c r="C29" s="15" t="inlineStr">
         <is>
           <t>2026-02-14</t>
         </is>
       </c>
-      <c r="D28" s="15" t="inlineStr"/>
-      <c r="E28" s="15" t="inlineStr">
+      <c r="D29" s="15" t="inlineStr"/>
+      <c r="E29" s="15" t="inlineStr">
         <is>
           <t>Accepted a different offer</t>
         </is>
@@ -1008,7 +1040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1044,6 +1076,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>